<commit_message>
feat(inventory): synchronize compound names with interactive maps, gazetteer and filters
</commit_message>
<xml_diff>
--- a/apps/sierra-estates-realty/public/downloads/Master_Inventory_Clean_No_Duplicates.xlsx
+++ b/apps/sierra-estates-realty/public/downloads/Master_Inventory_Clean_No_Duplicates.xlsx
@@ -566,7 +566,7 @@
         <v>OSA445</v>
       </c>
       <c r="B4" t="str">
-        <v>Eastown (SODIC)</v>
+        <v>Eastown</v>
       </c>
       <c r="C4" t="str">
         <v>New Cairo</v>
@@ -1043,7 +1043,7 @@
         <v>OSA540</v>
       </c>
       <c r="B13" t="str">
-        <v>Eastown (SODIC)</v>
+        <v>Eastown</v>
       </c>
       <c r="C13" t="str">
         <v>New Cairo</v>
@@ -1202,7 +1202,7 @@
         <v>OOA775</v>
       </c>
       <c r="B16" t="str">
-        <v>Oriana (CFC)</v>
+        <v>Oriana</v>
       </c>
       <c r="C16" t="str">
         <v>New Cairo</v>
@@ -3004,7 +3004,7 @@
         <v>OMM577</v>
       </c>
       <c r="B50" t="str">
-        <v>other</v>
+        <v>New Cairo</v>
       </c>
       <c r="C50" t="str">
         <v>New Cairo</v>
@@ -10954,7 +10954,7 @@
         <v>NC-3F-7.6M</v>
       </c>
       <c r="B200" t="str">
-        <v>other</v>
+        <v>New Cairo</v>
       </c>
       <c r="C200" t="str">
         <v>New Cairo</v>
@@ -12809,7 +12809,7 @@
         <v>SET-2B-140M-110K</v>
       </c>
       <c r="B235" t="str">
-        <v>Eastown (SODIC)</v>
+        <v>Eastown</v>
       </c>
       <c r="C235" t="str">
         <v>New Cairo</v>
@@ -14717,7 +14717,7 @@
         <v>REH-FR-2192</v>
       </c>
       <c r="B271" t="str">
-        <v>Eastown (SODIC)</v>
+        <v>Eastown</v>
       </c>
       <c r="C271" t="str">
         <v>New Cairo</v>
@@ -15539,7 +15539,7 @@
         <v>OSA540</v>
       </c>
       <c r="B6" t="str">
-        <v>Eastown (SODIC)</v>
+        <v>Eastown</v>
       </c>
       <c r="C6" t="str">
         <v>Apartment</v>
@@ -19564,7 +19564,7 @@
         <v>SET-2B-140M-110K</v>
       </c>
       <c r="B121" t="str">
-        <v>Eastown (SODIC)</v>
+        <v>Eastown</v>
       </c>
       <c r="C121" t="str">
         <v>Apartment</v>
@@ -20839,7 +20839,7 @@
         <v>NC-3F-7.6M</v>
       </c>
       <c r="B14" t="str">
-        <v>other</v>
+        <v>New Cairo</v>
       </c>
       <c r="C14" t="str">
         <v>Apartment</v>

</xml_diff>